<commit_message>
Updated player character properties
</commit_message>
<xml_diff>
--- a/_docs/CactusClan_trading.xlsx
+++ b/_docs/CactusClan_trading.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="383">
   <si>
     <t>Clan</t>
   </si>
@@ -724,9 +724,6 @@
     <t>Low speed; Overconfident; Vulnerable to fire</t>
   </si>
   <si>
-    <t>1000-2499</t>
-  </si>
-  <si>
     <t>Oasis Sovereign</t>
   </si>
   <si>
@@ -739,9 +736,6 @@
     <t>High mana cost; Targeted by enemies; Needs allies</t>
   </si>
   <si>
-    <t>2500+</t>
-  </si>
-  <si>
     <t>Tidestrider</t>
   </si>
   <si>
@@ -766,9 +760,6 @@
     <t>Low attack; Fragile; Needs protection</t>
   </si>
   <si>
-    <t>1500-2499</t>
-  </si>
-  <si>
     <t>Dunesoverlord</t>
   </si>
   <si>
@@ -1049,13 +1040,133 @@
   </si>
   <si>
     <t>Low agility; Slow attack speed; High mana cost</t>
+  </si>
+  <si>
+    <t>Crystalline Clan</t>
+  </si>
+  <si>
+    <t>Shardling</t>
+  </si>
+  <si>
+    <t>A tiny fragment of potential. Curious and eager to grow.</t>
+  </si>
+  <si>
+    <t>Curious; Eager to learn; Quick to grow</t>
+  </si>
+  <si>
+    <t>Fragile; Inexperienced; Easily scattered</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>Gemling</t>
+  </si>
+  <si>
+    <t>Cuts with precision. Learns quickly and adapts to any challenge.</t>
+  </si>
+  <si>
+    <t>Quick learner; Adaptable; Precise</t>
+  </si>
+  <si>
+    <t>Lightly armored; Overconfident; Impulsive</t>
+  </si>
+  <si>
+    <t>Crystalguard</t>
+  </si>
+  <si>
+    <t>Strong and steadfast. Protects allies with unbreakable resolve.</t>
+  </si>
+  <si>
+    <t>Strong defense; Loyal; Unbreakable resolve</t>
+  </si>
+  <si>
+    <t>Slow to change; Heavily armored; Not easily swayed</t>
+  </si>
+  <si>
+    <t>210</t>
+  </si>
+  <si>
+    <t>Prismwarden</t>
+  </si>
+  <si>
+    <t>Harnesses the power of light. Commands the battlefield with strategy.</t>
+  </si>
+  <si>
+    <t>Power of light; Strategic mind; Inspires allies</t>
+  </si>
+  <si>
+    <t>High mana cost; Takes time to focus; Vulnerable while casting</t>
+  </si>
+  <si>
+    <t>330</t>
+  </si>
+  <si>
+    <t>Crystal Emperor</t>
+  </si>
+  <si>
+    <t>An eternal sovereign. Unbreakable, brilliant, and ruler of all minerals.</t>
+  </si>
+  <si>
+    <t>Unmatched power; Master of all minerals; Commands all</t>
+  </si>
+  <si>
+    <t>Very high mana cost; Few understand; Burden of leadership</t>
+  </si>
+  <si>
+    <t>500+</t>
+  </si>
+  <si>
+    <t>Prism Forge</t>
+  </si>
+  <si>
+    <t>Shaper of glory, forger of might. Transforms crystals into legendary armaments.</t>
+  </si>
+  <si>
+    <t>Master craftsman; Enhances equipment; Creates powerful gear</t>
+  </si>
+  <si>
+    <t>Requires rare materials; Vulnerable while forging; Defends poorly</t>
+  </si>
+  <si>
+    <t>260</t>
+  </si>
+  <si>
+    <t>Ancient Prismlord</t>
+  </si>
+  <si>
+    <t>A tyrant of thorns and stone. His reign is pain. His legacy, eternal.</t>
+  </si>
+  <si>
+    <t>Unyielding durability; Thorned retaliation; Terrifies enemies</t>
+  </si>
+  <si>
+    <t>Slow and relentless; Low mobility; Magic disrupts crystals</t>
+  </si>
+  <si>
+    <t>350</t>
+  </si>
+  <si>
+    <t>Celestial Pricklord</t>
+  </si>
+  <si>
+    <t>Born from stars, forged from void. He commands crystals, bends destinies, he is eternal.</t>
+  </si>
+  <si>
+    <t>Cosmic power; Destroys all obstacles; Controls the battlefield</t>
+  </si>
+  <si>
+    <t>Arrogant and overconfident; Bound by ancient oaths; Vulnerable to pure light</t>
+  </si>
+  <si>
+    <t>450</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -1073,6 +1184,11 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11.0"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1088,7 +1204,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1099,6 +1215,18 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1645,6 +1773,9 @@
       <c r="A10" s="3" t="s">
         <v>49</v>
       </c>
+      <c r="B10" s="4">
+        <v>1.0</v>
+      </c>
       <c r="C10" s="3" t="s">
         <v>50</v>
       </c>
@@ -1677,6 +1808,9 @@
       <c r="A11" s="3" t="s">
         <v>49</v>
       </c>
+      <c r="B11" s="4">
+        <v>2.0</v>
+      </c>
       <c r="C11" s="3" t="s">
         <v>54</v>
       </c>
@@ -1709,6 +1843,9 @@
       <c r="A12" s="3" t="s">
         <v>49</v>
       </c>
+      <c r="B12" s="4">
+        <v>3.0</v>
+      </c>
       <c r="C12" s="3" t="s">
         <v>58</v>
       </c>
@@ -1741,6 +1878,9 @@
       <c r="A13" s="3" t="s">
         <v>49</v>
       </c>
+      <c r="B13" s="4">
+        <v>4.0</v>
+      </c>
       <c r="C13" s="3" t="s">
         <v>62</v>
       </c>
@@ -1773,6 +1913,9 @@
       <c r="A14" s="3" t="s">
         <v>49</v>
       </c>
+      <c r="B14" s="4">
+        <v>5.0</v>
+      </c>
       <c r="C14" s="3" t="s">
         <v>66</v>
       </c>
@@ -1805,6 +1948,9 @@
       <c r="A15" s="3" t="s">
         <v>49</v>
       </c>
+      <c r="B15" s="4">
+        <v>6.0</v>
+      </c>
       <c r="C15" s="3" t="s">
         <v>70</v>
       </c>
@@ -1837,6 +1983,9 @@
       <c r="A16" s="3" t="s">
         <v>49</v>
       </c>
+      <c r="B16" s="4">
+        <v>7.0</v>
+      </c>
       <c r="C16" s="3" t="s">
         <v>74</v>
       </c>
@@ -1869,6 +2018,9 @@
       <c r="A17" s="3" t="s">
         <v>49</v>
       </c>
+      <c r="B17" s="4">
+        <v>8.0</v>
+      </c>
       <c r="C17" s="3" t="s">
         <v>78</v>
       </c>
@@ -1901,6 +2053,9 @@
       <c r="A18" s="3" t="s">
         <v>82</v>
       </c>
+      <c r="B18" s="4">
+        <v>1.0</v>
+      </c>
       <c r="C18" s="3" t="s">
         <v>83</v>
       </c>
@@ -1933,6 +2088,9 @@
       <c r="A19" s="3" t="s">
         <v>82</v>
       </c>
+      <c r="B19" s="4">
+        <v>2.0</v>
+      </c>
       <c r="C19" s="3" t="s">
         <v>87</v>
       </c>
@@ -1965,6 +2123,9 @@
       <c r="A20" s="3" t="s">
         <v>82</v>
       </c>
+      <c r="B20" s="4">
+        <v>3.0</v>
+      </c>
       <c r="C20" s="3" t="s">
         <v>89</v>
       </c>
@@ -1997,6 +2158,9 @@
       <c r="A21" s="3" t="s">
         <v>82</v>
       </c>
+      <c r="B21" s="4">
+        <v>4.0</v>
+      </c>
       <c r="C21" s="3" t="s">
         <v>91</v>
       </c>
@@ -2029,6 +2193,9 @@
       <c r="A22" s="3" t="s">
         <v>82</v>
       </c>
+      <c r="B22" s="4">
+        <v>5.0</v>
+      </c>
       <c r="C22" s="3" t="s">
         <v>94</v>
       </c>
@@ -2061,6 +2228,9 @@
       <c r="A23" s="3" t="s">
         <v>82</v>
       </c>
+      <c r="B23" s="4">
+        <v>6.0</v>
+      </c>
       <c r="C23" s="3" t="s">
         <v>97</v>
       </c>
@@ -2093,6 +2263,9 @@
       <c r="A24" s="3" t="s">
         <v>82</v>
       </c>
+      <c r="B24" s="4">
+        <v>7.0</v>
+      </c>
       <c r="C24" s="3" t="s">
         <v>101</v>
       </c>
@@ -2125,6 +2298,9 @@
       <c r="A25" s="3" t="s">
         <v>82</v>
       </c>
+      <c r="B25" s="4">
+        <v>8.0</v>
+      </c>
       <c r="C25" s="3" t="s">
         <v>105</v>
       </c>
@@ -2157,6 +2333,9 @@
       <c r="A26" s="3" t="s">
         <v>109</v>
       </c>
+      <c r="B26" s="4">
+        <v>1.0</v>
+      </c>
       <c r="C26" s="3" t="s">
         <v>110</v>
       </c>
@@ -2189,6 +2368,9 @@
       <c r="A27" s="3" t="s">
         <v>109</v>
       </c>
+      <c r="B27" s="4">
+        <v>2.0</v>
+      </c>
       <c r="C27" s="3" t="s">
         <v>115</v>
       </c>
@@ -2221,6 +2403,9 @@
       <c r="A28" s="3" t="s">
         <v>109</v>
       </c>
+      <c r="B28" s="4">
+        <v>3.0</v>
+      </c>
       <c r="C28" s="3" t="s">
         <v>120</v>
       </c>
@@ -2253,6 +2438,9 @@
       <c r="A29" s="3" t="s">
         <v>109</v>
       </c>
+      <c r="B29" s="4">
+        <v>4.0</v>
+      </c>
       <c r="C29" s="3" t="s">
         <v>125</v>
       </c>
@@ -2285,6 +2473,9 @@
       <c r="A30" s="3" t="s">
         <v>109</v>
       </c>
+      <c r="B30" s="4">
+        <v>5.0</v>
+      </c>
       <c r="C30" s="3" t="s">
         <v>130</v>
       </c>
@@ -2317,6 +2508,9 @@
       <c r="A31" s="3" t="s">
         <v>109</v>
       </c>
+      <c r="B31" s="4">
+        <v>6.0</v>
+      </c>
       <c r="C31" s="3" t="s">
         <v>135</v>
       </c>
@@ -2349,6 +2543,9 @@
       <c r="A32" s="3" t="s">
         <v>109</v>
       </c>
+      <c r="B32" s="4">
+        <v>7.0</v>
+      </c>
       <c r="C32" s="3" t="s">
         <v>140</v>
       </c>
@@ -2381,6 +2578,9 @@
       <c r="A33" s="3" t="s">
         <v>109</v>
       </c>
+      <c r="B33" s="4">
+        <v>8.0</v>
+      </c>
       <c r="C33" s="3" t="s">
         <v>145</v>
       </c>
@@ -2413,6 +2613,9 @@
       <c r="A34" s="3" t="s">
         <v>150</v>
       </c>
+      <c r="B34" s="4">
+        <v>1.0</v>
+      </c>
       <c r="C34" s="3" t="s">
         <v>151</v>
       </c>
@@ -2445,6 +2648,9 @@
       <c r="A35" s="3" t="s">
         <v>150</v>
       </c>
+      <c r="B35" s="4">
+        <v>2.0</v>
+      </c>
       <c r="C35" s="3" t="s">
         <v>155</v>
       </c>
@@ -2477,6 +2683,9 @@
       <c r="A36" s="3" t="s">
         <v>150</v>
       </c>
+      <c r="B36" s="4">
+        <v>3.0</v>
+      </c>
       <c r="C36" s="3" t="s">
         <v>160</v>
       </c>
@@ -2509,6 +2718,9 @@
       <c r="A37" s="3" t="s">
         <v>150</v>
       </c>
+      <c r="B37" s="4">
+        <v>4.0</v>
+      </c>
       <c r="C37" s="3" t="s">
         <v>165</v>
       </c>
@@ -2541,6 +2753,9 @@
       <c r="A38" s="3" t="s">
         <v>150</v>
       </c>
+      <c r="B38" s="4">
+        <v>5.0</v>
+      </c>
       <c r="C38" s="3" t="s">
         <v>169</v>
       </c>
@@ -2573,6 +2788,9 @@
       <c r="A39" s="3" t="s">
         <v>150</v>
       </c>
+      <c r="B39" s="4">
+        <v>6.0</v>
+      </c>
       <c r="C39" s="3" t="s">
         <v>173</v>
       </c>
@@ -2605,6 +2823,9 @@
       <c r="A40" s="3" t="s">
         <v>150</v>
       </c>
+      <c r="B40" s="4">
+        <v>7.0</v>
+      </c>
       <c r="C40" s="3" t="s">
         <v>177</v>
       </c>
@@ -2637,6 +2858,9 @@
       <c r="A41" s="3" t="s">
         <v>150</v>
       </c>
+      <c r="B41" s="4">
+        <v>8.0</v>
+      </c>
       <c r="C41" s="3" t="s">
         <v>182</v>
       </c>
@@ -2669,6 +2893,9 @@
       <c r="A42" s="3" t="s">
         <v>186</v>
       </c>
+      <c r="B42" s="4">
+        <v>1.0</v>
+      </c>
       <c r="C42" s="3" t="s">
         <v>187</v>
       </c>
@@ -2701,6 +2928,9 @@
       <c r="A43" s="3" t="s">
         <v>186</v>
       </c>
+      <c r="B43" s="4">
+        <v>2.0</v>
+      </c>
       <c r="C43" s="3" t="s">
         <v>191</v>
       </c>
@@ -2733,6 +2963,9 @@
       <c r="A44" s="3" t="s">
         <v>186</v>
       </c>
+      <c r="B44" s="4">
+        <v>3.0</v>
+      </c>
       <c r="C44" s="3" t="s">
         <v>195</v>
       </c>
@@ -2765,6 +2998,9 @@
       <c r="A45" s="3" t="s">
         <v>186</v>
       </c>
+      <c r="B45" s="4">
+        <v>4.0</v>
+      </c>
       <c r="C45" s="3" t="s">
         <v>199</v>
       </c>
@@ -2797,6 +3033,9 @@
       <c r="A46" s="3" t="s">
         <v>186</v>
       </c>
+      <c r="B46" s="4">
+        <v>5.0</v>
+      </c>
       <c r="C46" s="3" t="s">
         <v>203</v>
       </c>
@@ -2829,6 +3068,9 @@
       <c r="A47" s="3" t="s">
         <v>186</v>
       </c>
+      <c r="B47" s="4">
+        <v>6.0</v>
+      </c>
       <c r="C47" s="3" t="s">
         <v>207</v>
       </c>
@@ -2861,6 +3103,9 @@
       <c r="A48" s="3" t="s">
         <v>186</v>
       </c>
+      <c r="B48" s="4">
+        <v>7.0</v>
+      </c>
       <c r="C48" s="3" t="s">
         <v>211</v>
       </c>
@@ -2893,6 +3138,9 @@
       <c r="A49" s="3" t="s">
         <v>186</v>
       </c>
+      <c r="B49" s="4">
+        <v>8.0</v>
+      </c>
       <c r="C49" s="3" t="s">
         <v>215</v>
       </c>
@@ -2925,6 +3173,9 @@
       <c r="A50" s="3" t="s">
         <v>220</v>
       </c>
+      <c r="B50" s="4">
+        <v>1.0</v>
+      </c>
       <c r="C50" s="3" t="s">
         <v>221</v>
       </c>
@@ -2957,6 +3208,9 @@
       <c r="A51" s="3" t="s">
         <v>220</v>
       </c>
+      <c r="B51" s="4">
+        <v>2.0</v>
+      </c>
       <c r="C51" s="3" t="s">
         <v>225</v>
       </c>
@@ -2989,6 +3243,9 @@
       <c r="A52" s="3" t="s">
         <v>220</v>
       </c>
+      <c r="B52" s="4">
+        <v>3.0</v>
+      </c>
       <c r="C52" s="3" t="s">
         <v>229</v>
       </c>
@@ -3021,6 +3278,9 @@
       <c r="A53" s="3" t="s">
         <v>220</v>
       </c>
+      <c r="B53" s="4">
+        <v>4.0</v>
+      </c>
       <c r="C53" s="3" t="s">
         <v>233</v>
       </c>
@@ -3045,25 +3305,28 @@
       <c r="J53" s="3">
         <v>80.0</v>
       </c>
-      <c r="K53" s="3" t="s">
-        <v>237</v>
+      <c r="K53" s="4">
+        <v>220.0</v>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="3" t="s">
         <v>220</v>
       </c>
+      <c r="B54" s="4">
+        <v>5.0</v>
+      </c>
       <c r="C54" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="D54" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="D54" s="3" t="s">
+      <c r="E54" s="3" t="s">
         <v>239</v>
       </c>
-      <c r="E54" s="3" t="s">
+      <c r="F54" s="3" t="s">
         <v>240</v>
-      </c>
-      <c r="F54" s="3" t="s">
-        <v>241</v>
       </c>
       <c r="G54" s="3">
         <v>95.0</v>
@@ -3077,25 +3340,28 @@
       <c r="J54" s="3">
         <v>100.0</v>
       </c>
-      <c r="K54" s="3" t="s">
-        <v>242</v>
+      <c r="K54" s="4">
+        <v>250.0</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="3" t="s">
         <v>220</v>
       </c>
+      <c r="B55" s="4">
+        <v>6.0</v>
+      </c>
       <c r="C55" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="E55" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="D55" s="3" t="s">
+      <c r="F55" s="3" t="s">
         <v>244</v>
-      </c>
-      <c r="E55" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="F55" s="3" t="s">
-        <v>246</v>
       </c>
       <c r="G55" s="3">
         <v>70.0</v>
@@ -3117,17 +3383,20 @@
       <c r="A56" s="3" t="s">
         <v>220</v>
       </c>
+      <c r="B56" s="4">
+        <v>7.0</v>
+      </c>
       <c r="C56" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="E56" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="D56" s="3" t="s">
+      <c r="F56" s="3" t="s">
         <v>248</v>
-      </c>
-      <c r="E56" s="3" t="s">
-        <v>249</v>
-      </c>
-      <c r="F56" s="3" t="s">
-        <v>250</v>
       </c>
       <c r="G56" s="3">
         <v>40.0</v>
@@ -3141,25 +3410,28 @@
       <c r="J56" s="3">
         <v>70.0</v>
       </c>
-      <c r="K56" s="3" t="s">
-        <v>251</v>
+      <c r="K56" s="4">
+        <v>400.0</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="3" t="s">
         <v>220</v>
       </c>
+      <c r="B57" s="4">
+        <v>8.0</v>
+      </c>
       <c r="C57" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="F57" s="3" t="s">
         <v>252</v>
-      </c>
-      <c r="D57" s="3" t="s">
-        <v>253</v>
-      </c>
-      <c r="E57" s="3" t="s">
-        <v>254</v>
-      </c>
-      <c r="F57" s="3" t="s">
-        <v>255</v>
       </c>
       <c r="G57" s="3">
         <v>95.0</v>
@@ -3174,24 +3446,27 @@
         <v>100.0</v>
       </c>
       <c r="K57" s="3" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="B58" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="E58" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="C58" s="3" t="s">
+      <c r="F58" s="3" t="s">
         <v>258</v>
-      </c>
-      <c r="D58" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="E58" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="F58" s="3" t="s">
-        <v>261</v>
       </c>
       <c r="G58" s="3">
         <v>10.0</v>
@@ -3211,19 +3486,22 @@
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="3" t="s">
-        <v>257</v>
+        <v>254</v>
+      </c>
+      <c r="B59" s="4">
+        <v>2.0</v>
       </c>
       <c r="C59" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="F59" s="3" t="s">
         <v>262</v>
-      </c>
-      <c r="D59" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="E59" s="3" t="s">
-        <v>264</v>
-      </c>
-      <c r="F59" s="3" t="s">
-        <v>265</v>
       </c>
       <c r="G59" s="3">
         <v>20.0</v>
@@ -3243,19 +3521,22 @@
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="3" t="s">
-        <v>257</v>
+        <v>254</v>
+      </c>
+      <c r="B60" s="4">
+        <v>3.0</v>
       </c>
       <c r="C60" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="F60" s="3" t="s">
         <v>266</v>
-      </c>
-      <c r="D60" s="3" t="s">
-        <v>267</v>
-      </c>
-      <c r="E60" s="3" t="s">
-        <v>268</v>
-      </c>
-      <c r="F60" s="3" t="s">
-        <v>269</v>
       </c>
       <c r="G60" s="3">
         <v>40.0</v>
@@ -3275,19 +3556,22 @@
     </row>
     <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="3" t="s">
-        <v>257</v>
+        <v>254</v>
+      </c>
+      <c r="B61" s="4">
+        <v>4.0</v>
       </c>
       <c r="C61" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="F61" s="3" t="s">
         <v>270</v>
-      </c>
-      <c r="D61" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="E61" s="3" t="s">
-        <v>272</v>
-      </c>
-      <c r="F61" s="3" t="s">
-        <v>273</v>
       </c>
       <c r="G61" s="3">
         <v>30.0</v>
@@ -3307,19 +3591,22 @@
     </row>
     <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="3" t="s">
-        <v>257</v>
+        <v>254</v>
+      </c>
+      <c r="B62" s="4">
+        <v>5.0</v>
       </c>
       <c r="C62" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="F62" s="3" t="s">
         <v>274</v>
-      </c>
-      <c r="D62" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="E62" s="3" t="s">
-        <v>276</v>
-      </c>
-      <c r="F62" s="3" t="s">
-        <v>277</v>
       </c>
       <c r="G62" s="3">
         <v>35.0</v>
@@ -3339,19 +3626,22 @@
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="3" t="s">
-        <v>257</v>
+        <v>254</v>
+      </c>
+      <c r="B63" s="4">
+        <v>6.0</v>
       </c>
       <c r="C63" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="F63" s="3" t="s">
         <v>278</v>
-      </c>
-      <c r="D63" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="E63" s="3" t="s">
-        <v>280</v>
-      </c>
-      <c r="F63" s="3" t="s">
-        <v>281</v>
       </c>
       <c r="G63" s="3">
         <v>50.0</v>
@@ -3371,19 +3661,22 @@
     </row>
     <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="3" t="s">
-        <v>257</v>
+        <v>254</v>
+      </c>
+      <c r="B64" s="4">
+        <v>7.0</v>
       </c>
       <c r="C64" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="E64" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="F64" s="3" t="s">
         <v>282</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="E64" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="F64" s="3" t="s">
-        <v>285</v>
       </c>
       <c r="G64" s="3">
         <v>70.0</v>
@@ -3403,19 +3696,22 @@
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="3" t="s">
-        <v>257</v>
+        <v>254</v>
+      </c>
+      <c r="B65" s="4">
+        <v>8.0</v>
       </c>
       <c r="C65" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="E65" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="F65" s="3" t="s">
         <v>286</v>
-      </c>
-      <c r="D65" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="E65" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="F65" s="3" t="s">
-        <v>289</v>
       </c>
       <c r="G65" s="3">
         <v>90.0</v>
@@ -3435,19 +3731,22 @@
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="B66" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E66" s="3" t="s">
         <v>290</v>
       </c>
-      <c r="C66" s="3" t="s">
+      <c r="F66" s="3" t="s">
         <v>291</v>
-      </c>
-      <c r="D66" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="E66" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="F66" s="3" t="s">
-        <v>294</v>
       </c>
       <c r="G66" s="3">
         <v>10.0</v>
@@ -3462,24 +3761,27 @@
         <v>20.0</v>
       </c>
       <c r="K66" s="3" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="3" t="s">
-        <v>290</v>
+        <v>287</v>
+      </c>
+      <c r="B67" s="4">
+        <v>2.0</v>
       </c>
       <c r="C67" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="F67" s="3" t="s">
         <v>296</v>
-      </c>
-      <c r="D67" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="E67" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="F67" s="3" t="s">
-        <v>299</v>
       </c>
       <c r="G67" s="3">
         <v>25.0</v>
@@ -3499,19 +3801,22 @@
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="3" t="s">
-        <v>290</v>
+        <v>287</v>
+      </c>
+      <c r="B68" s="4">
+        <v>3.0</v>
       </c>
       <c r="C68" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="F68" s="3" t="s">
         <v>300</v>
-      </c>
-      <c r="D68" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="E68" s="3" t="s">
-        <v>302</v>
-      </c>
-      <c r="F68" s="3" t="s">
-        <v>303</v>
       </c>
       <c r="G68" s="3">
         <v>60.0</v>
@@ -3526,24 +3831,27 @@
         <v>60.0</v>
       </c>
       <c r="K68" s="3" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="3" t="s">
-        <v>290</v>
+        <v>287</v>
+      </c>
+      <c r="B69" s="4">
+        <v>4.0</v>
       </c>
       <c r="C69" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="F69" s="3" t="s">
         <v>305</v>
-      </c>
-      <c r="D69" s="3" t="s">
-        <v>306</v>
-      </c>
-      <c r="E69" s="3" t="s">
-        <v>307</v>
-      </c>
-      <c r="F69" s="3" t="s">
-        <v>308</v>
       </c>
       <c r="G69" s="3">
         <v>85.0</v>
@@ -3563,19 +3871,22 @@
     </row>
     <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="3" t="s">
-        <v>290</v>
+        <v>287</v>
+      </c>
+      <c r="B70" s="4">
+        <v>5.0</v>
       </c>
       <c r="C70" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="F70" s="3" t="s">
         <v>309</v>
-      </c>
-      <c r="D70" s="3" t="s">
-        <v>310</v>
-      </c>
-      <c r="E70" s="3" t="s">
-        <v>311</v>
-      </c>
-      <c r="F70" s="3" t="s">
-        <v>312</v>
       </c>
       <c r="G70" s="3">
         <v>95.0</v>
@@ -3590,24 +3901,27 @@
         <v>90.0</v>
       </c>
       <c r="K70" s="3" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="3" t="s">
-        <v>290</v>
+        <v>287</v>
+      </c>
+      <c r="B71" s="4">
+        <v>6.0</v>
       </c>
       <c r="C71" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="F71" s="3" t="s">
         <v>314</v>
-      </c>
-      <c r="D71" s="3" t="s">
-        <v>315</v>
-      </c>
-      <c r="E71" s="3" t="s">
-        <v>316</v>
-      </c>
-      <c r="F71" s="3" t="s">
-        <v>317</v>
       </c>
       <c r="G71" s="3">
         <v>70.0</v>
@@ -3627,19 +3941,22 @@
     </row>
     <row r="72" ht="15.75" customHeight="1">
       <c r="A72" s="3" t="s">
-        <v>290</v>
+        <v>287</v>
+      </c>
+      <c r="B72" s="4">
+        <v>7.0</v>
       </c>
       <c r="C72" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="F72" s="3" t="s">
         <v>318</v>
-      </c>
-      <c r="D72" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="E72" s="3" t="s">
-        <v>320</v>
-      </c>
-      <c r="F72" s="3" t="s">
-        <v>321</v>
       </c>
       <c r="G72" s="3">
         <v>80.0</v>
@@ -3659,19 +3976,22 @@
     </row>
     <row r="73" ht="15.75" customHeight="1">
       <c r="A73" s="3" t="s">
-        <v>290</v>
+        <v>287</v>
+      </c>
+      <c r="B73" s="4">
+        <v>8.0</v>
       </c>
       <c r="C73" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="E73" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="F73" s="3" t="s">
         <v>322</v>
-      </c>
-      <c r="D73" s="3" t="s">
-        <v>323</v>
-      </c>
-      <c r="E73" s="3" t="s">
-        <v>324</v>
-      </c>
-      <c r="F73" s="3" t="s">
-        <v>325</v>
       </c>
       <c r="G73" s="3">
         <v>30.0</v>
@@ -3691,13 +4011,16 @@
     </row>
     <row r="74" ht="15.75" customHeight="1">
       <c r="A74" s="3" t="s">
-        <v>326</v>
+        <v>323</v>
+      </c>
+      <c r="B74" s="4">
+        <v>1.0</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="E74" s="3" t="s">
         <v>85</v>
@@ -3723,13 +4046,16 @@
     </row>
     <row r="75" ht="15.75" customHeight="1">
       <c r="A75" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="B75" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="C75" s="3" t="s">
         <v>326</v>
       </c>
-      <c r="C75" s="3" t="s">
-        <v>329</v>
-      </c>
       <c r="D75" s="3" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="E75" s="3" t="s">
         <v>14</v>
@@ -3755,13 +4081,16 @@
     </row>
     <row r="76" ht="15.75" customHeight="1">
       <c r="A76" s="3" t="s">
-        <v>326</v>
+        <v>323</v>
+      </c>
+      <c r="B76" s="4">
+        <v>3.0</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="E76" s="3" t="s">
         <v>24</v>
@@ -3787,13 +4116,16 @@
     </row>
     <row r="77" ht="15.75" customHeight="1">
       <c r="A77" s="3" t="s">
-        <v>326</v>
+        <v>323</v>
+      </c>
+      <c r="B77" s="4">
+        <v>4.0</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="E77" s="3" t="s">
         <v>43</v>
@@ -3819,13 +4151,16 @@
     </row>
     <row r="78" ht="15.75" customHeight="1">
       <c r="A78" s="3" t="s">
-        <v>326</v>
+        <v>323</v>
+      </c>
+      <c r="B78" s="4">
+        <v>5.0</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="E78" s="3" t="s">
         <v>47</v>
@@ -3851,13 +4186,16 @@
     </row>
     <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="3" t="s">
-        <v>326</v>
+        <v>323</v>
+      </c>
+      <c r="B79" s="4">
+        <v>6.0</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="E79" s="3" t="s">
         <v>33</v>
@@ -3883,16 +4221,19 @@
     </row>
     <row r="80" ht="15.75" customHeight="1">
       <c r="A80" s="3" t="s">
-        <v>326</v>
+        <v>323</v>
+      </c>
+      <c r="B80" s="4">
+        <v>7.0</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="E80" s="3" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="F80" s="3" t="s">
         <v>108</v>
@@ -3915,19 +4256,22 @@
     </row>
     <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="3" t="s">
-        <v>326</v>
+        <v>323</v>
+      </c>
+      <c r="B81" s="4">
+        <v>8.0</v>
       </c>
       <c r="C81" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="E81" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="F81" s="3" t="s">
         <v>342</v>
-      </c>
-      <c r="D81" s="3" t="s">
-        <v>343</v>
-      </c>
-      <c r="E81" s="3" t="s">
-        <v>344</v>
-      </c>
-      <c r="F81" s="3" t="s">
-        <v>345</v>
       </c>
       <c r="G81" s="3">
         <v>90.0</v>
@@ -3945,14 +4289,286 @@
         <v>399.0</v>
       </c>
     </row>
-    <row r="82" ht="15.75" customHeight="1"/>
-    <row r="83" ht="15.75" customHeight="1"/>
-    <row r="84" ht="15.75" customHeight="1"/>
-    <row r="85" ht="15.75" customHeight="1"/>
-    <row r="86" ht="15.75" customHeight="1"/>
-    <row r="87" ht="15.75" customHeight="1"/>
-    <row r="88" ht="15.75" customHeight="1"/>
-    <row r="89" ht="15.75" customHeight="1"/>
+    <row r="82" ht="15.75" customHeight="1">
+      <c r="A82" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="B82" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="C82" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="D82" s="5" t="s">
+        <v>345</v>
+      </c>
+      <c r="E82" s="7" t="s">
+        <v>346</v>
+      </c>
+      <c r="F82" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="G82" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="H82" s="8">
+        <v>10.0</v>
+      </c>
+      <c r="I82" s="8">
+        <v>25.0</v>
+      </c>
+      <c r="J82" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="K82" s="7" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="83" ht="15.75" customHeight="1">
+      <c r="A83" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="B83" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="C83" s="7" t="s">
+        <v>349</v>
+      </c>
+      <c r="D83" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="E83" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="F83" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="G83" s="8">
+        <v>25.0</v>
+      </c>
+      <c r="H83" s="8">
+        <v>20.0</v>
+      </c>
+      <c r="I83" s="8">
+        <v>50.0</v>
+      </c>
+      <c r="J83" s="8">
+        <v>35.0</v>
+      </c>
+      <c r="K83" s="7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="84" ht="15.75" customHeight="1">
+      <c r="A84" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="B84" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="C84" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="D84" s="7" t="s">
+        <v>354</v>
+      </c>
+      <c r="E84" s="7" t="s">
+        <v>355</v>
+      </c>
+      <c r="F84" s="7" t="s">
+        <v>356</v>
+      </c>
+      <c r="G84" s="8">
+        <v>45.0</v>
+      </c>
+      <c r="H84" s="8">
+        <v>70.0</v>
+      </c>
+      <c r="I84" s="8">
+        <v>30.0</v>
+      </c>
+      <c r="J84" s="8">
+        <v>80.0</v>
+      </c>
+      <c r="K84" s="7" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="85" ht="15.75" customHeight="1">
+      <c r="A85" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="B85" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="C85" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="D85" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="E85" s="7" t="s">
+        <v>360</v>
+      </c>
+      <c r="F85" s="7" t="s">
+        <v>361</v>
+      </c>
+      <c r="G85" s="8">
+        <v>70.0</v>
+      </c>
+      <c r="H85" s="8">
+        <v>60.0</v>
+      </c>
+      <c r="I85" s="8">
+        <v>40.0</v>
+      </c>
+      <c r="J85" s="8">
+        <v>90.0</v>
+      </c>
+      <c r="K85" s="7" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="86" ht="15.75" customHeight="1">
+      <c r="A86" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="B86" s="6">
+        <v>5.0</v>
+      </c>
+      <c r="C86" s="7" t="s">
+        <v>363</v>
+      </c>
+      <c r="D86" s="7" t="s">
+        <v>364</v>
+      </c>
+      <c r="E86" s="7" t="s">
+        <v>365</v>
+      </c>
+      <c r="F86" s="7" t="s">
+        <v>366</v>
+      </c>
+      <c r="G86" s="8">
+        <v>95.0</v>
+      </c>
+      <c r="H86" s="8">
+        <v>90.0</v>
+      </c>
+      <c r="I86" s="8">
+        <v>50.0</v>
+      </c>
+      <c r="J86" s="8">
+        <v>120.0</v>
+      </c>
+      <c r="K86" s="7" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="87" ht="15.75" customHeight="1">
+      <c r="A87" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="B87" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="C87" s="7" t="s">
+        <v>368</v>
+      </c>
+      <c r="D87" s="7" t="s">
+        <v>369</v>
+      </c>
+      <c r="E87" s="7" t="s">
+        <v>370</v>
+      </c>
+      <c r="F87" s="7" t="s">
+        <v>371</v>
+      </c>
+      <c r="G87" s="8">
+        <v>60.0</v>
+      </c>
+      <c r="H87" s="8">
+        <v>80.0</v>
+      </c>
+      <c r="I87" s="8">
+        <v>40.0</v>
+      </c>
+      <c r="J87" s="8">
+        <v>100.0</v>
+      </c>
+      <c r="K87" s="7" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="88" ht="15.75" customHeight="1">
+      <c r="A88" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="B88" s="6">
+        <v>7.0</v>
+      </c>
+      <c r="C88" s="7" t="s">
+        <v>373</v>
+      </c>
+      <c r="D88" s="7" t="s">
+        <v>374</v>
+      </c>
+      <c r="E88" s="7" t="s">
+        <v>375</v>
+      </c>
+      <c r="F88" s="7" t="s">
+        <v>376</v>
+      </c>
+      <c r="G88" s="8">
+        <v>85.0</v>
+      </c>
+      <c r="H88" s="8">
+        <v>110.0</v>
+      </c>
+      <c r="I88" s="8">
+        <v>25.0</v>
+      </c>
+      <c r="J88" s="8">
+        <v>130.0</v>
+      </c>
+      <c r="K88" s="7" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="89" ht="15.75" customHeight="1">
+      <c r="A89" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="B89" s="6">
+        <v>8.0</v>
+      </c>
+      <c r="C89" s="7" t="s">
+        <v>378</v>
+      </c>
+      <c r="D89" s="7" t="s">
+        <v>379</v>
+      </c>
+      <c r="E89" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="F89" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="G89" s="8">
+        <v>110.0</v>
+      </c>
+      <c r="H89" s="8">
+        <v>120.0</v>
+      </c>
+      <c r="I89" s="8">
+        <v>35.0</v>
+      </c>
+      <c r="J89" s="8">
+        <v>140.0</v>
+      </c>
+      <c r="K89" s="7" t="s">
+        <v>382</v>
+      </c>
+    </row>
     <row r="90" ht="15.75" customHeight="1"/>
     <row r="91" ht="15.75" customHeight="1"/>
     <row r="92" ht="15.75" customHeight="1"/>

</xml_diff>